<commit_message>
added batch module post request and created batchId
</commit_message>
<xml_diff>
--- a/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
+++ b/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/Documents/Maya Numpy Ninja/APIRestAssuredLMSHackathon/Team03_Restful_Ninjas_LMS_Hackathon/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saphi\eclipse-workspace\Team03_RestfulNinjas_LMS_Hackathon\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23943D14-2ECD-7745-9EED-8861CD8A0D6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{600F8852-7C8D-4CDD-9193-018425FE2F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="94">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -63,12 +63,6 @@
   </si>
   <si>
     <t>Ok</t>
-  </si>
-  <si>
-    <t>CreateBatch_Valid_batchName</t>
-  </si>
-  <si>
-    <t>/batches</t>
   </si>
   <si>
     <t>{
@@ -84,15 +78,6 @@
 }</t>
   </si>
   <si>
-    <t>{
-"batchDescription": "test description",
-"batchName": "javarogrammijjjng_12",
-"batchNoOfClasses": 1,
-"batchStatus": "Active",
-"programId": ""
-}</t>
-  </si>
-  <si>
     <t>Valid credential</t>
   </si>
   <si>
@@ -338,12 +323,48 @@
   <si>
     <t>{"programDescription": "PPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPP", "programName": "Prog Java", "programStatus": "Active"}</t>
   </si>
+  <si>
+    <t>batchName</t>
+  </si>
+  <si>
+    <t>batchDescription</t>
+  </si>
+  <si>
+    <t>batchStatus</t>
+  </si>
+  <si>
+    <t>batchNoOfClasses</t>
+  </si>
+  <si>
+    <t>expectedStatus</t>
+  </si>
+  <si>
+    <t>expectedMessage</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Batch created</t>
+  </si>
+  <si>
+    <t>Mandatory_Optional_Valid</t>
+  </si>
+  <si>
+    <t>P3185_B01</t>
+  </si>
+  <si>
+    <t>ValidBatchDescription</t>
+  </si>
+  <si>
+    <t>/batches</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -389,21 +410,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color rgb="FF0451A5"/>
       <name val="IBMPlexMono"/>
@@ -419,6 +425,13 @@
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="IBMPlexMono"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -468,7 +481,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -486,29 +499,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -526,6 +517,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -745,141 +746,141 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F999"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="44.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.1640625" customWidth="1"/>
+    <col min="2" max="2" width="44.796875" customWidth="1"/>
+    <col min="3" max="3" width="32.1328125" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
     <col min="5" max="5" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="27" t="s">
+      <c r="E1" s="15" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="17">
+        <v>200</v>
+      </c>
+      <c r="E2" s="15"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A3" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="17">
+        <v>404</v>
+      </c>
+      <c r="E3" s="15"/>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A4" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="27" t="s">
+      <c r="B4" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="29">
-        <v>200</v>
-      </c>
-      <c r="E2" s="27"/>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A3" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="27" t="s">
+      <c r="D4" s="17">
+        <v>415</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A5" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="29">
-        <v>404</v>
-      </c>
-      <c r="E3" s="27"/>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A4" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="27" t="s">
+      <c r="D5" s="17">
+        <v>401</v>
+      </c>
+      <c r="E5" s="15"/>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A6" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="29">
-        <v>415</v>
-      </c>
-      <c r="E4" s="27" t="s">
+      <c r="D6" s="17">
+        <v>400</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A5" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="27" t="s">
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A7" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="29">
-        <v>401</v>
-      </c>
-      <c r="E5" s="27"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A6" s="27" t="s">
+      <c r="B7" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="28" t="s">
+      <c r="C7" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="17">
+        <v>400</v>
+      </c>
+      <c r="E7" s="15" t="s">
         <v>26</v>
-      </c>
-      <c r="C6" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="29">
-        <v>400</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A7" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="29">
-        <v>400</v>
-      </c>
-      <c r="E7" s="27" t="s">
-        <v>29</v>
       </c>
       <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="30" t="s">
-        <v>32</v>
+        <v>27</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>29</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>5</v>
@@ -887,17 +888,17 @@
       <c r="D8" s="2">
         <v>400</v>
       </c>
-      <c r="E8" s="27" t="s">
-        <v>29</v>
+      <c r="E8" s="15" t="s">
+        <v>26</v>
       </c>
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>33</v>
+        <v>28</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>30</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>5</v>
@@ -905,14 +906,14 @@
       <c r="D9" s="2">
         <v>200</v>
       </c>
-      <c r="E9" s="27"/>
+      <c r="E9" s="15"/>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="30" t="s">
-        <v>36</v>
+        <v>34</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>33</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>5</v>
@@ -921,16 +922,16 @@
         <v>400</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="30" t="s">
-        <v>46</v>
+        <v>35</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>5</v>
@@ -938,17 +939,17 @@
       <c r="D11" s="2">
         <v>400</v>
       </c>
-      <c r="E11" s="27" t="s">
-        <v>47</v>
+      <c r="E11" s="15" t="s">
+        <v>44</v>
       </c>
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="30" t="s">
-        <v>40</v>
+        <v>36</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>37</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>5</v>
@@ -957,16 +958,16 @@
         <v>401</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" s="30" t="s">
-        <v>42</v>
+        <v>38</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>39</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>5</v>
@@ -975,16 +976,16 @@
         <v>400</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B14" s="30" t="s">
-        <v>48</v>
+        <v>40</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>5</v>
@@ -992,17 +993,17 @@
       <c r="D14" s="2">
         <v>400</v>
       </c>
-      <c r="E14" s="27" t="s">
-        <v>29</v>
+      <c r="E14" s="15" t="s">
+        <v>26</v>
       </c>
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B15" s="30" t="s">
-        <v>14</v>
+        <v>42</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>12</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>5</v>
@@ -1011,19 +1012,19 @@
         <v>405</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="30" t="s">
-        <v>60</v>
+        <v>52</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>57</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D16" s="2">
         <v>201</v>
@@ -1033,112 +1034,112 @@
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" s="30" t="s">
-        <v>60</v>
+        <v>53</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>57</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D17" s="2">
         <v>404</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F17" s="1"/>
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" s="30" t="s">
-        <v>61</v>
+        <v>59</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>58</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D18" s="2">
         <v>400</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F18" s="1"/>
     </row>
     <row r="19" spans="1:6" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D19" s="2">
         <v>400</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F19" s="1"/>
     </row>
     <row r="20" spans="1:6" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D20" s="2">
         <v>400</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F20" s="1"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B21" s="30" t="s">
-        <v>60</v>
+        <v>56</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>57</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D21" s="2">
         <v>415</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F21" s="1"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B22" s="30" t="s">
-        <v>65</v>
+        <v>63</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>62</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D22" s="2">
         <v>401</v>
       </c>
       <c r="E22" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
@@ -2200,33 +2201,33 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Z1008"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="62.83203125" customWidth="1"/>
-    <col min="2" max="2" width="93.1640625" customWidth="1"/>
+    <col min="1" max="1" width="62.796875" customWidth="1"/>
+    <col min="2" max="2" width="93.1328125" customWidth="1"/>
     <col min="3" max="3" width="38.33203125" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G1" s="5"/>
@@ -2251,34 +2252,34 @@
       <c r="Z1" s="5"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="24" t="s">
+      <c r="B2" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="25">
+      <c r="E2" s="13">
         <v>201</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="12" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="15.75" customHeight="1">
       <c r="A3" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>10</v>
@@ -2287,35 +2288,35 @@
         <v>404</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E4" s="7">
         <v>405</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>9</v>
@@ -2327,15 +2328,15 @@
         <v>400</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>9</v>
@@ -2347,15 +2348,15 @@
         <v>400</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="15.75" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>9</v>
@@ -2367,15 +2368,15 @@
         <v>400</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="15.75" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>9</v>
@@ -2387,32 +2388,32 @@
         <v>400</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A9" s="16"/>
-      <c r="B9" s="26"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A10" s="16"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A11" s="16"/>
-      <c r="B11" s="26"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1">
       <c r="A12" s="7"/>
@@ -3824,325 +3825,169 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F1014"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:H1014"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="42.1640625" customWidth="1"/>
-    <col min="2" max="2" width="47.33203125" customWidth="1"/>
-    <col min="3" max="3" width="28.6640625" customWidth="1"/>
-    <col min="4" max="4" width="21.5" customWidth="1"/>
-    <col min="5" max="5" width="32" customWidth="1"/>
+    <col min="1" max="1" width="22.3984375" customWidth="1"/>
+    <col min="2" max="2" width="30.3984375" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" customWidth="1"/>
+    <col min="4" max="4" width="14.3984375" customWidth="1"/>
+    <col min="5" max="6" width="17.73046875" customWidth="1"/>
+    <col min="7" max="7" width="18.86328125" customWidth="1"/>
+    <col min="8" max="8" width="18.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:8" ht="12.75">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="14" t="s">
+      <c r="B1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="17"/>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A2" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="19">
+      <c r="G1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="12.75">
+      <c r="A2" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2">
         <v>201</v>
       </c>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A3" s="15"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A5" s="15"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A6" s="16"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A7" s="15"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="17"/>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A8" s="15"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="17"/>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A9" s="15"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A10" s="15"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-    </row>
-    <row r="11" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A11" s="15"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A12" s="15"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="17"/>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A13" s="15"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="17"/>
-    </row>
-    <row r="14" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A14" s="15"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="17"/>
-    </row>
-    <row r="15" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A15" s="15"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="17"/>
-    </row>
-    <row r="16" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A16" s="15"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="17"/>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A17" s="15"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="17"/>
-    </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A18" s="16"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A19" s="16"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-    </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-    </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A21" s="16"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-    </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A22" s="16"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="16"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="17"/>
-    </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A24" s="16"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A25" s="16"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-    </row>
+      <c r="H2" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="12.75"/>
+    <row r="4" spans="1:8" ht="12.75"/>
+    <row r="5" spans="1:8" ht="12.75"/>
+    <row r="6" spans="1:8" ht="12.75"/>
+    <row r="7" spans="1:8" ht="12.75"/>
+    <row r="8" spans="1:8" ht="12.75"/>
+    <row r="9" spans="1:8" ht="12.75"/>
+    <row r="10" spans="1:8" ht="12.75"/>
+    <row r="11" spans="1:8" ht="12.75"/>
+    <row r="12" spans="1:8" ht="12.75"/>
+    <row r="13" spans="1:8" ht="12.75"/>
+    <row r="14" spans="1:8" ht="12.75"/>
+    <row r="15" spans="1:8" ht="12.75"/>
+    <row r="16" spans="1:8" ht="12.75"/>
+    <row r="17" spans="1:6" ht="12.75"/>
+    <row r="18" spans="1:6" ht="12.75"/>
+    <row r="19" spans="1:6" ht="12.75"/>
+    <row r="20" spans="1:6" ht="12.75"/>
+    <row r="21" spans="1:6" ht="12.75"/>
+    <row r="22" spans="1:6" ht="12.75"/>
+    <row r="23" spans="1:6" ht="12.75"/>
+    <row r="24" spans="1:6" ht="12.75"/>
+    <row r="25" spans="1:6" ht="12.75"/>
     <row r="26" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A26" s="16"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="16"/>
+      <c r="A26" s="7"/>
+      <c r="C26" s="7"/>
       <c r="D26" s="19"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A27" s="16"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="16"/>
+      <c r="A27" s="7"/>
+      <c r="C27" s="7"/>
       <c r="D27" s="19"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="17"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A28" s="16"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="16"/>
+      <c r="A28" s="7"/>
+      <c r="C28" s="7"/>
       <c r="D28" s="19"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
     </row>
     <row r="29" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A29" s="16"/>
-      <c r="B29" s="17"/>
-      <c r="C29" s="16"/>
+      <c r="A29" s="7"/>
+      <c r="C29" s="7"/>
       <c r="D29" s="19"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A30" s="16"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="16"/>
+      <c r="A30" s="7"/>
+      <c r="C30" s="7"/>
       <c r="D30" s="19"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="17"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A31" s="16"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="16"/>
+      <c r="A31" s="7"/>
+      <c r="C31" s="7"/>
       <c r="D31" s="19"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
     </row>
     <row r="32" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A32" s="16"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="16"/>
+      <c r="A32" s="7"/>
+      <c r="C32" s="7"/>
       <c r="D32" s="19"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
     </row>
     <row r="33" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A33" s="16"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
     </row>
     <row r="34" spans="1:6" ht="15.75" customHeight="1">
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
-      <c r="E34" s="11"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
     </row>
     <row r="35" spans="1:6" ht="15.75" customHeight="1">
       <c r="A35" s="7"/>
       <c r="B35" s="7"/>
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="11"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1">
       <c r="A36" s="7"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="11"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
     </row>
     <row r="37" spans="1:6" ht="15.75" customHeight="1">
       <c r="A37" s="7"/>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
-      <c r="E37" s="11"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1">
       <c r="A38" s="7"/>
@@ -4161,7 +4006,8 @@
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
-      <c r="E40" s="11"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="21"/>
     </row>
     <row r="41" spans="1:6" ht="15.75" customHeight="1">
       <c r="A41" s="7"/>
@@ -4174,90 +4020,97 @@
       <c r="B42" s="7"/>
       <c r="C42" s="7"/>
       <c r="D42" s="7"/>
-      <c r="E42" s="11"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="21"/>
     </row>
     <row r="43" spans="1:6" ht="15.75" customHeight="1">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
       <c r="C43" s="7"/>
       <c r="D43" s="7"/>
-      <c r="E43" s="11"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="21"/>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
-      <c r="E44" s="11"/>
+      <c r="E44" s="21"/>
+      <c r="F44" s="21"/>
     </row>
     <row r="45" spans="1:6" ht="15.75" customHeight="1">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
-      <c r="E45" s="11"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
     </row>
     <row r="46" spans="1:6" ht="15.75" customHeight="1">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
-      <c r="E46" s="12"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
     </row>
     <row r="47" spans="1:6" ht="15.75" customHeight="1">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
-      <c r="E47" s="12"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
     </row>
     <row r="48" spans="1:6" ht="15.75" customHeight="1">
       <c r="A48" s="7"/>
       <c r="C48" s="7"/>
       <c r="D48" s="7"/>
     </row>
-    <row r="49" spans="1:5" ht="15.75" customHeight="1">
+    <row r="49" spans="1:6" ht="15.75" customHeight="1">
       <c r="A49" s="7"/>
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
     </row>
-    <row r="50" spans="1:5" ht="15.75" customHeight="1">
+    <row r="50" spans="1:6" ht="15.75" customHeight="1">
       <c r="A50" s="7"/>
       <c r="C50" s="7"/>
       <c r="D50" s="7"/>
     </row>
-    <row r="51" spans="1:5" ht="15.75" customHeight="1">
+    <row r="51" spans="1:6" ht="15.75" customHeight="1">
       <c r="A51" s="7"/>
       <c r="C51" s="7"/>
       <c r="D51" s="7"/>
-      <c r="E51" s="13"/>
-    </row>
-    <row r="52" spans="1:5" ht="15.75" customHeight="1">
+      <c r="E51" s="23"/>
+      <c r="F51" s="23"/>
+    </row>
+    <row r="52" spans="1:6" ht="15.75" customHeight="1">
       <c r="A52" s="7"/>
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
     </row>
-    <row r="53" spans="1:5" ht="15.75" customHeight="1">
+    <row r="53" spans="1:6" ht="15.75" customHeight="1">
       <c r="A53" s="7"/>
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
     </row>
-    <row r="54" spans="1:5" ht="15.75" customHeight="1">
+    <row r="54" spans="1:6" ht="15.75" customHeight="1">
       <c r="A54" s="7"/>
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
     </row>
-    <row r="55" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="56" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="57" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="58" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="59" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="60" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="61" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="62" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="63" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="64" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="55" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="56" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="57" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="58" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="59" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="60" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="61" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="62" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="63" spans="1:6" ht="15.75" customHeight="1"/>
+    <row r="64" spans="1:6" ht="15.75" customHeight="1"/>
     <row r="65" ht="15.75" customHeight="1"/>
     <row r="66" ht="15.75" customHeight="1"/>
     <row r="67" ht="15.75" customHeight="1"/>
@@ -5210,5 +5063,6 @@
     <row r="1014" ht="15.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added Batch module Post scenarios
</commit_message>
<xml_diff>
--- a/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
+++ b/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saphi\eclipse-workspace\Team03_RestfulNinjas_LMS_Hackathon\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{600F8852-7C8D-4CDD-9193-018425FE2F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D33C9E29-D73D-409C-9006-AEE1720E2FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5745" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="174">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -345,26 +345,266 @@
     <t>Active</t>
   </si>
   <si>
-    <t>Batch created</t>
-  </si>
-  <si>
-    <t>Mandatory_Optional_Valid</t>
-  </si>
-  <si>
-    <t>P3185_B01</t>
-  </si>
-  <si>
-    <t>ValidBatchDescription</t>
-  </si>
-  <si>
     <t>/batches</t>
+  </si>
+  <si>
+    <t>programId</t>
+  </si>
+  <si>
+    <t>programName</t>
+  </si>
+  <si>
+    <t>Mandatory_Optional_Fields</t>
+  </si>
+  <si>
+    <t>Mandatory_Only_Fields</t>
+  </si>
+  <si>
+    <t>Optional_Only_Fields</t>
+  </si>
+  <si>
+    <t>ProgramName_Mismatch</t>
+  </si>
+  <si>
+    <t>Inactive_ProgramId</t>
+  </si>
+  <si>
+    <t>ProgramId_NotExist</t>
+  </si>
+  <si>
+    <t>BatchName_No_Underscore</t>
+  </si>
+  <si>
+    <t>BatchName_Hyphen</t>
+  </si>
+  <si>
+    <t>BatchName_Char_Suffix</t>
+  </si>
+  <si>
+    <t>BatchName_Special_Suffix</t>
+  </si>
+  <si>
+    <t>BatchName_Too_Long</t>
+  </si>
+  <si>
+    <t>BatchName_Too_Short</t>
+  </si>
+  <si>
+    <t>BatchName_Duplicate</t>
+  </si>
+  <si>
+    <t>Description_Too_Short</t>
+  </si>
+  <si>
+    <t>Description_Too_Long</t>
+  </si>
+  <si>
+    <t>Status_Random_Chars</t>
+  </si>
+  <si>
+    <t>Status_Numbers</t>
+  </si>
+  <si>
+    <t>Status_Special</t>
+  </si>
+  <si>
+    <t>Classes_NonNumeric</t>
+  </si>
+  <si>
+    <t>Classes_Too_Small</t>
+  </si>
+  <si>
+    <t>Classes_Too_Large</t>
+  </si>
+  <si>
+    <t>Invalid_Endpoint</t>
+  </si>
+  <si>
+    <t>Invalid_Method</t>
+  </si>
+  <si>
+    <t>Invalid_ContentType</t>
+  </si>
+  <si>
+    <t>No_Authorization</t>
+  </si>
+  <si>
+    <t>ValidDesc</t>
+  </si>
+  <si>
+    <t>Abc</t>
+  </si>
+  <si>
+    <t>ThisDescriptionIsWayTooLongToBeValid</t>
+  </si>
+  <si>
+    <t>abc</t>
+  </si>
+  <si>
+    <t>Valid POST</t>
+  </si>
+  <si>
+    <t>Missing mandatory fields</t>
+  </si>
+  <si>
+    <t>API overrides programName</t>
+  </si>
+  <si>
+    <t>Program inactive</t>
+  </si>
+  <si>
+    <t>Program not found</t>
+  </si>
+  <si>
+    <t>Missing underscore</t>
+  </si>
+  <si>
+    <t>Hyphen not allowed</t>
+  </si>
+  <si>
+    <t>Suffix must be numeric</t>
+  </si>
+  <si>
+    <t>Special char not allowed</t>
+  </si>
+  <si>
+    <t>&gt; 28 chars</t>
+  </si>
+  <si>
+    <t>&lt; 6 chars</t>
+  </si>
+  <si>
+    <t>Duplicate name</t>
+  </si>
+  <si>
+    <t>&lt; 4 chars</t>
+  </si>
+  <si>
+    <t>&gt; 25 chars</t>
+  </si>
+  <si>
+    <t>Invalid status</t>
+  </si>
+  <si>
+    <t>Non-numeric</t>
+  </si>
+  <si>
+    <t>&lt; 1</t>
+  </si>
+  <si>
+    <t>&gt; 99</t>
+  </si>
+  <si>
+    <t>Wrong endpoint</t>
+  </si>
+  <si>
+    <t>Wrong method</t>
+  </si>
+  <si>
+    <t>Wrong content type</t>
+  </si>
+  <si>
+    <t>Missing token</t>
+  </si>
+  <si>
+    <t>PUT</t>
+  </si>
+  <si>
+    <t>_1</t>
+  </si>
+  <si>
+    <t>_2</t>
+  </si>
+  <si>
+    <t>_3</t>
+  </si>
+  <si>
+    <t>_4</t>
+  </si>
+  <si>
+    <t>_5</t>
+  </si>
+  <si>
+    <t>_6</t>
+  </si>
+  <si>
+    <t>_a</t>
+  </si>
+  <si>
+    <t>_@</t>
+  </si>
+  <si>
+    <t>_123456789012345678901234567890</t>
+  </si>
+  <si>
+    <t>_13</t>
+  </si>
+  <si>
+    <t>_15</t>
+  </si>
+  <si>
+    <t>_16</t>
+  </si>
+  <si>
+    <t>_17</t>
+  </si>
+  <si>
+    <t>_18</t>
+  </si>
+  <si>
+    <t>_19</t>
+  </si>
+  <si>
+    <t>_20</t>
+  </si>
+  <si>
+    <t>_21</t>
+  </si>
+  <si>
+    <t>_22</t>
+  </si>
+  <si>
+    <t>_23</t>
+  </si>
+  <si>
+    <t>_24</t>
+  </si>
+  <si>
+    <t>_25</t>
+  </si>
+  <si>
+    <t>_26</t>
+  </si>
+  <si>
+    <t>RandomChars</t>
+  </si>
+  <si>
+    <t>@@@</t>
+  </si>
+  <si>
+    <t>contentType</t>
+  </si>
+  <si>
+    <t>authorization</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>ValidDesc InvalidConentType</t>
+  </si>
+  <si>
+    <t>rJtkPqKy</t>
+  </si>
+  <si>
+    <t>plain</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -433,6 +673,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -478,10 +732,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -517,18 +772,31 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3825,292 +4093,1002 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H1014"/>
+  <dimension ref="A1:M1014"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="22.3984375" customWidth="1"/>
-    <col min="2" max="2" width="30.3984375" customWidth="1"/>
-    <col min="3" max="3" width="27.33203125" customWidth="1"/>
-    <col min="4" max="4" width="14.3984375" customWidth="1"/>
-    <col min="5" max="6" width="17.73046875" customWidth="1"/>
-    <col min="7" max="7" width="18.86328125" customWidth="1"/>
-    <col min="8" max="8" width="18.796875" customWidth="1"/>
+    <col min="1" max="1" width="22.3984375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="35.19921875" style="20" customWidth="1"/>
+    <col min="3" max="3" width="33.06640625" style="19" customWidth="1"/>
+    <col min="4" max="4" width="14.3984375" style="19" customWidth="1"/>
+    <col min="5" max="7" width="17.73046875" style="19" customWidth="1"/>
+    <col min="8" max="8" width="18.86328125" style="19" customWidth="1"/>
+    <col min="9" max="9" width="25.46484375" style="19" customWidth="1"/>
+    <col min="10" max="16384" width="12.6640625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="12.75">
-      <c r="A1" t="s">
+    <row r="1" spans="1:13" ht="12.75">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" s="19" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="12.75">
-      <c r="A2" s="24" t="s">
+      <c r="J1" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="K1" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="L1" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="M1" s="21" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="12.75">
+      <c r="A2" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="B2" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D2" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="19">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G2" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="19">
+        <v>201</v>
+      </c>
+      <c r="I2" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="12.75">
+      <c r="A3" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="G2">
+      <c r="B3" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3" s="19">
+        <v>5</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="19">
         <v>201</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="I3" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="13.9" customHeight="1">
+      <c r="A4" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="F4" s="19" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="12.75"/>
-    <row r="4" spans="1:8" ht="12.75"/>
-    <row r="5" spans="1:8" ht="12.75"/>
-    <row r="6" spans="1:8" ht="12.75"/>
-    <row r="7" spans="1:8" ht="12.75"/>
-    <row r="8" spans="1:8" ht="12.75"/>
-    <row r="9" spans="1:8" ht="12.75"/>
-    <row r="10" spans="1:8" ht="12.75"/>
-    <row r="11" spans="1:8" ht="12.75"/>
-    <row r="12" spans="1:8" ht="12.75"/>
-    <row r="13" spans="1:8" ht="12.75"/>
-    <row r="14" spans="1:8" ht="12.75"/>
-    <row r="15" spans="1:8" ht="12.75"/>
-    <row r="16" spans="1:8" ht="12.75"/>
-    <row r="17" spans="1:6" ht="12.75"/>
-    <row r="18" spans="1:6" ht="12.75"/>
-    <row r="19" spans="1:6" ht="12.75"/>
-    <row r="20" spans="1:6" ht="12.75"/>
-    <row r="21" spans="1:6" ht="12.75"/>
-    <row r="22" spans="1:6" ht="12.75"/>
-    <row r="23" spans="1:6" ht="12.75"/>
-    <row r="24" spans="1:6" ht="12.75"/>
-    <row r="25" spans="1:6" ht="12.75"/>
-    <row r="26" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="19"/>
-    </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-    </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="19"/>
-    </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A29" s="7"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="19"/>
-    </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A30" s="7"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
-    </row>
-    <row r="31" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="19"/>
-    </row>
-    <row r="32" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A32" s="7"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="19"/>
-    </row>
-    <row r="33" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-    </row>
-    <row r="34" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
-    </row>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-    </row>
-    <row r="36" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
-    </row>
-    <row r="37" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A37" s="7"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="21"/>
-    </row>
-    <row r="38" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A38" s="7"/>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-    </row>
-    <row r="39" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A39" s="7"/>
-      <c r="B39" s="7"/>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7"/>
-    </row>
-    <row r="40" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A40" s="7"/>
-      <c r="B40" s="7"/>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
-    </row>
-    <row r="41" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A41" s="7"/>
-      <c r="B41" s="7"/>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7"/>
-    </row>
-    <row r="42" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A42" s="7"/>
-      <c r="B42" s="7"/>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
-      <c r="E42" s="21"/>
-      <c r="F42" s="21"/>
-    </row>
-    <row r="43" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A43" s="7"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="21"/>
-      <c r="F43" s="21"/>
-    </row>
-    <row r="44" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A44" s="7"/>
-      <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="21"/>
-      <c r="F44" s="21"/>
-    </row>
-    <row r="45" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A45" s="7"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="7"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="21"/>
-      <c r="F45" s="21"/>
-    </row>
-    <row r="46" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A46" s="7"/>
-      <c r="B46" s="7"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
-    </row>
-    <row r="47" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A47" s="7"/>
-      <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-    </row>
-    <row r="48" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A48" s="7"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="7"/>
-    </row>
-    <row r="49" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A49" s="7"/>
-      <c r="C49" s="7"/>
-      <c r="D49" s="7"/>
-    </row>
-    <row r="50" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-    </row>
-    <row r="51" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A51" s="7"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="23"/>
-      <c r="F51" s="23"/>
-    </row>
-    <row r="52" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A52" s="7"/>
-      <c r="C52" s="7"/>
-      <c r="D52" s="7"/>
-    </row>
-    <row r="53" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A53" s="7"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
-    </row>
-    <row r="54" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A54" s="7"/>
-      <c r="B54" s="7"/>
-      <c r="C54" s="7"/>
-      <c r="D54" s="7"/>
-    </row>
-    <row r="55" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="56" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="57" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="58" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="59" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="60" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="61" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="62" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="63" spans="1:6" ht="15.75" customHeight="1"/>
-    <row r="64" spans="1:6" ht="15.75" customHeight="1"/>
+      <c r="G4" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="19">
+        <v>400</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="12.75">
+      <c r="A5" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" s="19">
+        <v>10</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="19">
+        <v>201</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="K5" s="21" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="12.75">
+      <c r="A6" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E6" s="19">
+        <v>10</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="19">
+        <v>400</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="J6" s="19">
+        <v>3110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="12.75">
+      <c r="A7" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E7" s="19">
+        <v>10</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="19">
+        <v>404</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="J7" s="19">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="12.75">
+      <c r="A8" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="20">
+        <v>7</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" s="19">
+        <v>10</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" s="19">
+        <v>400</v>
+      </c>
+      <c r="I8" s="19" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="12.75">
+      <c r="A9" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="20">
+        <v>-8</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="19">
+        <v>10</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" s="19">
+        <v>400</v>
+      </c>
+      <c r="I9" s="19" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="12.75">
+      <c r="A10" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E10" s="19">
+        <v>10</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" s="19">
+        <v>400</v>
+      </c>
+      <c r="I10" s="19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="12.75">
+      <c r="A11" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" s="19">
+        <v>10</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" s="19">
+        <v>400</v>
+      </c>
+      <c r="I11" s="19" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="12.75">
+      <c r="A12" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E12" s="19">
+        <v>10</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G12" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" s="19">
+        <v>400</v>
+      </c>
+      <c r="I12" s="19" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="12.75">
+      <c r="A13" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" s="19">
+        <v>10</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" s="19">
+        <v>400</v>
+      </c>
+      <c r="I13" s="19" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="12.75">
+      <c r="A14" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E14" s="19">
+        <v>10</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" s="19">
+        <v>400</v>
+      </c>
+      <c r="I14" s="19" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="12.75">
+      <c r="A15" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="19">
+        <v>10</v>
+      </c>
+      <c r="F15" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="19">
+        <v>400</v>
+      </c>
+      <c r="I15" s="19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="12.75">
+      <c r="A16" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16" s="19">
+        <v>10</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" s="19">
+        <v>400</v>
+      </c>
+      <c r="I16" s="19" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="12.75">
+      <c r="A17" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>166</v>
+      </c>
+      <c r="E17" s="19">
+        <v>10</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" s="19">
+        <v>400</v>
+      </c>
+      <c r="I17" s="19" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="12.75">
+      <c r="A18" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D18" s="22">
+        <v>12345</v>
+      </c>
+      <c r="E18" s="19">
+        <v>10</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H18" s="19">
+        <v>400</v>
+      </c>
+      <c r="I18" s="19" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="12.75">
+      <c r="A19" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="E19" s="19">
+        <v>10</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" s="19">
+        <v>400</v>
+      </c>
+      <c r="I19" s="19" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="12.75">
+      <c r="A20" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E20" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="F20" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" s="19">
+        <v>400</v>
+      </c>
+      <c r="I20" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="12.75">
+      <c r="A21" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E21" s="19">
+        <v>0</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G21" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H21" s="19">
+        <v>400</v>
+      </c>
+      <c r="I21" s="19" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="12.75">
+      <c r="A22" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E22" s="19">
+        <v>100</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G22" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H22" s="19">
+        <v>400</v>
+      </c>
+      <c r="I22" s="19" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="12.75">
+      <c r="A23" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E23" s="19">
+        <v>10</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" s="19">
+        <v>404</v>
+      </c>
+      <c r="I23" s="19" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="12.75">
+      <c r="A24" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E24" s="19">
+        <v>10</v>
+      </c>
+      <c r="F24" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G24" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="H24" s="19">
+        <v>405</v>
+      </c>
+      <c r="I24" s="19" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="12.75">
+      <c r="A25" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>171</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E25" s="19">
+        <v>10</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G25" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H25" s="19">
+        <v>415</v>
+      </c>
+      <c r="I25" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="L25" s="21" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="15.75" customHeight="1">
+      <c r="A26" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E26" s="19">
+        <v>10</v>
+      </c>
+      <c r="F26" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G26" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" s="19">
+        <v>401</v>
+      </c>
+      <c r="I26" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="M26" s="21" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="15.75" customHeight="1">
+      <c r="A27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+    </row>
+    <row r="28" spans="1:13" ht="15.75" customHeight="1">
+      <c r="A28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="26"/>
+    </row>
+    <row r="29" spans="1:13" ht="15.75" customHeight="1">
+      <c r="A29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="26"/>
+    </row>
+    <row r="30" spans="1:13" ht="15.75" customHeight="1">
+      <c r="A30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+    </row>
+    <row r="31" spans="1:13" ht="15.75" customHeight="1">
+      <c r="A31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="26"/>
+    </row>
+    <row r="32" spans="1:13" ht="15.75" customHeight="1">
+      <c r="A32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="26"/>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A33" s="25"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A34" s="25"/>
+      <c r="B34" s="26"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="28"/>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A35" s="25"/>
+      <c r="B35" s="26"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A36" s="25"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
+      <c r="G36" s="28"/>
+    </row>
+    <row r="37" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A37" s="25"/>
+      <c r="B37" s="26"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="28"/>
+    </row>
+    <row r="38" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A38" s="25"/>
+      <c r="B38" s="26"/>
+      <c r="C38" s="25"/>
+      <c r="D38" s="25"/>
+    </row>
+    <row r="39" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A39" s="25"/>
+      <c r="B39" s="26"/>
+      <c r="C39" s="25"/>
+      <c r="D39" s="25"/>
+    </row>
+    <row r="40" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A40" s="25"/>
+      <c r="B40" s="26"/>
+      <c r="C40" s="25"/>
+      <c r="D40" s="25"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
+    </row>
+    <row r="41" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A41" s="25"/>
+      <c r="B41" s="26"/>
+      <c r="C41" s="25"/>
+      <c r="D41" s="25"/>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A42" s="25"/>
+      <c r="B42" s="26"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A43" s="25"/>
+      <c r="B43" s="26"/>
+      <c r="C43" s="25"/>
+      <c r="D43" s="25"/>
+      <c r="E43" s="28"/>
+      <c r="F43" s="28"/>
+      <c r="G43" s="28"/>
+    </row>
+    <row r="44" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A44" s="25"/>
+      <c r="B44" s="26"/>
+      <c r="C44" s="25"/>
+      <c r="D44" s="25"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="28"/>
+      <c r="G44" s="28"/>
+    </row>
+    <row r="45" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A45" s="25"/>
+      <c r="B45" s="26"/>
+      <c r="C45" s="25"/>
+      <c r="D45" s="25"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="28"/>
+    </row>
+    <row r="46" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A46" s="25"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="25"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+    </row>
+    <row r="47" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A47" s="25"/>
+      <c r="B47" s="26"/>
+      <c r="C47" s="25"/>
+      <c r="D47" s="25"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="29"/>
+      <c r="G47" s="29"/>
+    </row>
+    <row r="48" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A48" s="25"/>
+      <c r="C48" s="25"/>
+      <c r="D48" s="25"/>
+    </row>
+    <row r="49" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A49" s="25"/>
+      <c r="C49" s="25"/>
+      <c r="D49" s="25"/>
+    </row>
+    <row r="50" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A50" s="25"/>
+      <c r="C50" s="25"/>
+      <c r="D50" s="25"/>
+    </row>
+    <row r="51" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A51" s="25"/>
+      <c r="C51" s="25"/>
+      <c r="D51" s="25"/>
+      <c r="E51" s="30"/>
+      <c r="F51" s="30"/>
+      <c r="G51" s="30"/>
+    </row>
+    <row r="52" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A52" s="25"/>
+      <c r="C52" s="25"/>
+      <c r="D52" s="25"/>
+    </row>
+    <row r="53" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A53" s="25"/>
+      <c r="C53" s="25"/>
+      <c r="D53" s="25"/>
+    </row>
+    <row r="54" spans="1:7" ht="15.75" customHeight="1">
+      <c r="A54" s="25"/>
+      <c r="B54" s="26"/>
+      <c r="C54" s="25"/>
+      <c r="D54" s="25"/>
+    </row>
+    <row r="55" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="56" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="57" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="58" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="59" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="60" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="61" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="62" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="63" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="64" spans="1:7" ht="15.75" customHeight="1"/>
     <row r="65" ht="15.75" customHeight="1"/>
     <row r="66" ht="15.75" customHeight="1"/>
     <row r="67" ht="15.75" customHeight="1"/>
@@ -5062,7 +6040,11 @@
     <row r="1013" ht="15.75" customHeight="1"/>
     <row r="1014" ht="15.75" customHeight="1"/>
   </sheetData>
+  <phoneticPr fontId="12" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B11" r:id="rId1" xr:uid="{53FA3B93-59E6-4995-AC4D-40A7B013FC6F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added Batch module Get All Batches
</commit_message>
<xml_diff>
--- a/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
+++ b/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maya/Documents/Maya Numpy Ninja/APIRestAssuredLMSHackathon/Team03_Restful_Ninjas_LMS_Hackathon/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saphi\eclipse-workspace\Team03_RestfulNinjas_LMS_Hackathon\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C8A98C6-E8F2-8C46-BAF2-57D7DCBDC822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B73967-63A5-4749-A222-61A362277A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5745" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="203">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -667,6 +667,27 @@
   </si>
   <si>
     <t>OK</t>
+  </si>
+  <si>
+    <t>py_</t>
+  </si>
+  <si>
+    <t>Get_all_Valid</t>
+  </si>
+  <si>
+    <t>Get_All_Invalid_EP</t>
+  </si>
+  <si>
+    <t>Get_All_Invalid_Method</t>
+  </si>
+  <si>
+    <t>Get_All_No_Auth</t>
+  </si>
+  <si>
+    <t>Method Not Allowed</t>
+  </si>
+  <si>
+    <t>Get_All_Invalid_ContentType</t>
   </si>
 </sst>
 </file>
@@ -805,7 +826,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -857,6 +878,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1077,11 +1099,11 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F998"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="44.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.1640625" customWidth="1"/>
+    <col min="2" max="2" width="44.796875" customWidth="1"/>
+    <col min="3" max="3" width="32.1328125" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
     <col min="5" max="5" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
@@ -2542,14 +2564,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Z1008"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="62.83203125" customWidth="1"/>
-    <col min="2" max="2" width="93.1640625" customWidth="1"/>
+    <col min="1" max="1" width="62.796875" customWidth="1"/>
+    <col min="2" max="2" width="93.1328125" customWidth="1"/>
     <col min="3" max="3" width="38.33203125" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1">
@@ -4244,18 +4266,20 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:M1014"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
-    <col min="2" max="2" width="35.1640625" style="17" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" style="17" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
     <col min="4" max="4" width="14.33203125" customWidth="1"/>
-    <col min="5" max="7" width="17.6640625" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="25.5" customWidth="1"/>
+    <col min="5" max="5" width="15.9296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.9296875" customWidth="1"/>
+    <col min="8" max="8" width="18.796875" customWidth="1"/>
+    <col min="9" max="9" width="25.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13">
+    <row r="1" spans="1:13" ht="12.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4296,7 +4320,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="13">
+    <row r="2" spans="1:13" ht="12.75">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -4325,7 +4349,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="13">
+    <row r="3" spans="1:13" ht="12.75">
       <c r="A3" t="s">
         <v>92</v>
       </c>
@@ -4377,7 +4401,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="13">
+    <row r="5" spans="1:13" ht="12.75">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -4409,7 +4433,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="13">
+    <row r="6" spans="1:13" ht="12.75">
       <c r="A6" s="18" t="s">
         <v>95</v>
       </c>
@@ -4441,7 +4465,7 @@
         <v>3110</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="13">
+    <row r="7" spans="1:13" ht="12.75">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -4473,7 +4497,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="13">
+    <row r="8" spans="1:13" ht="12.75">
       <c r="A8" s="18" t="s">
         <v>97</v>
       </c>
@@ -4502,7 +4526,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="13">
+    <row r="9" spans="1:13" ht="12.75">
       <c r="A9" t="s">
         <v>98</v>
       </c>
@@ -4531,7 +4555,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="13">
+    <row r="10" spans="1:13" ht="12.75">
       <c r="A10" t="s">
         <v>99</v>
       </c>
@@ -4560,7 +4584,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13">
+    <row r="11" spans="1:13" ht="12.75">
       <c r="A11" t="s">
         <v>100</v>
       </c>
@@ -4589,7 +4613,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="13">
+    <row r="12" spans="1:13" ht="12.75">
       <c r="A12" t="s">
         <v>101</v>
       </c>
@@ -4618,7 +4642,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="13">
+    <row r="13" spans="1:13" ht="12.75">
       <c r="A13" s="18" t="s">
         <v>102</v>
       </c>
@@ -4646,8 +4670,11 @@
       <c r="I13" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" ht="13">
+      <c r="K13" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="12.75">
       <c r="A14" t="s">
         <v>103</v>
       </c>
@@ -4676,7 +4703,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="13">
+    <row r="15" spans="1:13" ht="12.75">
       <c r="A15" t="s">
         <v>104</v>
       </c>
@@ -4705,7 +4732,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="13">
+    <row r="16" spans="1:13" ht="12.75">
       <c r="A16" t="s">
         <v>105</v>
       </c>
@@ -4734,7 +4761,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="13">
+    <row r="17" spans="1:13" ht="12.75">
       <c r="A17" t="s">
         <v>106</v>
       </c>
@@ -4763,7 +4790,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="13">
+    <row r="18" spans="1:13" ht="12.75">
       <c r="A18" t="s">
         <v>107</v>
       </c>
@@ -4792,7 +4819,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="13">
+    <row r="19" spans="1:13" ht="12.75">
       <c r="A19" t="s">
         <v>108</v>
       </c>
@@ -4821,7 +4848,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="13">
+    <row r="20" spans="1:13" ht="12.75">
       <c r="A20" t="s">
         <v>109</v>
       </c>
@@ -4850,7 +4877,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="13">
+    <row r="21" spans="1:13" ht="12.75">
       <c r="A21" t="s">
         <v>110</v>
       </c>
@@ -4879,7 +4906,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="13">
+    <row r="22" spans="1:13" ht="12.75">
       <c r="A22" t="s">
         <v>111</v>
       </c>
@@ -4908,7 +4935,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="13">
+    <row r="23" spans="1:13" ht="12.75">
       <c r="A23" s="18" t="s">
         <v>112</v>
       </c>
@@ -4937,7 +4964,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="13">
+    <row r="24" spans="1:13" ht="12.75">
       <c r="A24" t="s">
         <v>113</v>
       </c>
@@ -4966,7 +4993,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="13">
+    <row r="25" spans="1:13" ht="12.75">
       <c r="A25" t="s">
         <v>114</v>
       </c>
@@ -5031,35 +5058,107 @@
       </c>
     </row>
     <row r="27" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A27" s="6"/>
+      <c r="A27" s="6" t="s">
+        <v>197</v>
+      </c>
       <c r="C27" s="6"/>
       <c r="D27" s="22"/>
       <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
+      <c r="F27" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="G27" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="H27">
+        <v>200</v>
+      </c>
+      <c r="I27" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="28" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A28" s="6"/>
+      <c r="A28" s="6" t="s">
+        <v>198</v>
+      </c>
       <c r="C28" s="6"/>
       <c r="D28" s="22"/>
+      <c r="F28" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" t="s">
+        <v>65</v>
+      </c>
+      <c r="H28">
+        <v>404</v>
+      </c>
+      <c r="I28" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="29" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A29" s="6"/>
+      <c r="A29" s="6" t="s">
+        <v>199</v>
+      </c>
       <c r="C29" s="6"/>
       <c r="D29" s="22"/>
+      <c r="F29" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G29" t="s">
+        <v>142</v>
+      </c>
+      <c r="H29">
+        <v>405</v>
+      </c>
+      <c r="I29" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="30" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A30" s="6"/>
+      <c r="A30" s="6" t="s">
+        <v>200</v>
+      </c>
       <c r="C30" s="6"/>
       <c r="D30" s="22"/>
       <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
+      <c r="F30" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="H30">
+        <v>401</v>
+      </c>
+      <c r="I30" t="s">
+        <v>141</v>
+      </c>
+      <c r="M30" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="31" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A31" s="6"/>
+      <c r="A31" s="6" t="s">
+        <v>202</v>
+      </c>
       <c r="C31" s="6"/>
       <c r="D31" s="22"/>
+      <c r="F31" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="H31">
+        <v>415</v>
+      </c>
+      <c r="I31" t="s">
+        <v>140</v>
+      </c>
+      <c r="L31" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="32" spans="1:13" ht="15.75" customHeight="1">
       <c r="A32" s="6"/>

</xml_diff>

<commit_message>
Added Get Batch by Id scenario
</commit_message>
<xml_diff>
--- a/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
+++ b/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saphi\eclipse-workspace\Team03_RestfulNinjas_LMS_Hackathon\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B73967-63A5-4749-A222-61A362277A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC233BA-CB4A-40FE-8C56-0D16F738CDEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5745" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="206">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -689,12 +689,21 @@
   <si>
     <t>Get_All_Invalid_ContentType</t>
   </si>
+  <si>
+    <t>Get_Batch_By_Id_Valid</t>
+  </si>
+  <si>
+    <t>/batches/batchId/{batchId}</t>
+  </si>
+  <si>
+    <t>Valid Get Batch By Id</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -777,6 +786,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -826,7 +841,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -879,6 +894,7 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4268,12 +4284,12 @@
   <dimension ref="A1:M1014"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="22.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29" customWidth="1"/>
     <col min="2" max="2" width="22.33203125" style="17" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
     <col min="4" max="4" width="14.33203125" customWidth="1"/>
     <col min="5" max="5" width="15.9296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.6640625" customWidth="1"/>
+    <col min="6" max="6" width="29.796875" customWidth="1"/>
     <col min="7" max="7" width="13.9296875" customWidth="1"/>
     <col min="8" max="8" width="18.796875" customWidth="1"/>
     <col min="9" max="9" width="25.46484375" customWidth="1"/>
@@ -5161,9 +5177,23 @@
       </c>
     </row>
     <row r="32" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A32" s="6"/>
+      <c r="A32" s="28" t="s">
+        <v>203</v>
+      </c>
       <c r="C32" s="6"/>
       <c r="D32" s="22"/>
+      <c r="F32" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G32" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="H32">
+        <v>200</v>
+      </c>
+      <c r="I32" s="18" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="33" spans="1:7" ht="15.75" customHeight="1">
       <c r="A33" s="6"/>

</xml_diff>

<commit_message>
Added Get, Put, Delete batch scenarios for valid case
</commit_message>
<xml_diff>
--- a/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
+++ b/src/test/resources/Team3_Restful_Ninjas_TestDataSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saphi\eclipse-workspace\Team03_RestfulNinjas_LMS_Hackathon\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC233BA-CB4A-40FE-8C56-0D16F738CDEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{581F10E2-2A65-45DF-B735-6A8AFD0A21C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5745" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="219">
   <si>
     <t>ScenarioName</t>
   </si>
@@ -698,12 +698,51 @@
   <si>
     <t>Valid Get Batch By Id</t>
   </si>
+  <si>
+    <t>Get_Batch_By_Name_Valid</t>
+  </si>
+  <si>
+    <t>/batches/batchName/{batchName}</t>
+  </si>
+  <si>
+    <t>Get_Batch_By_ProgramId_Valid</t>
+  </si>
+  <si>
+    <t>Update_Batch_By_Id_Valid</t>
+  </si>
+  <si>
+    <t>Delete_Batch_By_Id_Valid</t>
+  </si>
+  <si>
+    <t>DELETE</t>
+  </si>
+  <si>
+    <t>/batches/{batchId}</t>
+  </si>
+  <si>
+    <t>/batches/{id}</t>
+  </si>
+  <si>
+    <t>/batches/program/{programId}</t>
+  </si>
+  <si>
+    <t>Valid Get Batch By Name</t>
+  </si>
+  <si>
+    <t>Valid Get Batch By ProgramId</t>
+  </si>
+  <si>
+    <t>Valid Put Batch By Id</t>
+  </si>
+  <si>
+    <t>Valid Delete Batch By Id</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -786,12 +825,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -841,7 +874,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -894,7 +927,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5177,7 +5209,7 @@
       </c>
     </row>
     <row r="32" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="6" t="s">
         <v>203</v>
       </c>
       <c r="C32" s="6"/>
@@ -5195,40 +5227,91 @@
         <v>205</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A33" s="6"/>
-      <c r="B33" s="22"/>
+    <row r="33" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A33" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>146</v>
+      </c>
       <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-    </row>
-    <row r="34" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A34" s="6"/>
-      <c r="B34" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="F33" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="H33">
+        <v>200</v>
+      </c>
+      <c r="I33" s="18" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A34" s="6" t="s">
+        <v>208</v>
+      </c>
       <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-    </row>
-    <row r="35" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A35" s="6"/>
-      <c r="B35" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="F34" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="H34">
+        <v>200</v>
+      </c>
+      <c r="I34" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A35" s="6" t="s">
+        <v>209</v>
+      </c>
       <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
-    </row>
-    <row r="36" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A36" s="6"/>
-      <c r="B36" s="22"/>
+      <c r="D35" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="H35">
+        <v>200</v>
+      </c>
+      <c r="I35" s="18" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A36" s="6" t="s">
+        <v>210</v>
+      </c>
       <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24"/>
-    </row>
-    <row r="37" spans="1:7" ht="15.75" customHeight="1">
+      <c r="D36" s="22"/>
+      <c r="F36" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="H36">
+        <v>200</v>
+      </c>
+      <c r="I36" s="18" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="15.75" customHeight="1">
       <c r="A37" s="6"/>
       <c r="B37" s="22"/>
       <c r="C37" s="6"/>
@@ -5237,19 +5320,19 @@
       <c r="F37" s="24"/>
       <c r="G37" s="24"/>
     </row>
-    <row r="38" spans="1:7" ht="15.75" customHeight="1">
+    <row r="38" spans="1:9" ht="15.75" customHeight="1">
       <c r="A38" s="6"/>
       <c r="B38" s="22"/>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
     </row>
-    <row r="39" spans="1:7" ht="15.75" customHeight="1">
+    <row r="39" spans="1:9" ht="15.75" customHeight="1">
       <c r="A39" s="6"/>
       <c r="B39" s="22"/>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
     </row>
-    <row r="40" spans="1:7" ht="15.75" customHeight="1">
+    <row r="40" spans="1:9" ht="15.75" customHeight="1">
       <c r="A40" s="6"/>
       <c r="B40" s="22"/>
       <c r="C40" s="6"/>
@@ -5258,13 +5341,13 @@
       <c r="F40" s="24"/>
       <c r="G40" s="24"/>
     </row>
-    <row r="41" spans="1:7" ht="15.75" customHeight="1">
+    <row r="41" spans="1:9" ht="15.75" customHeight="1">
       <c r="A41" s="6"/>
       <c r="B41" s="22"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
     </row>
-    <row r="42" spans="1:7" ht="15.75" customHeight="1">
+    <row r="42" spans="1:9" ht="15.75" customHeight="1">
       <c r="A42" s="6"/>
       <c r="B42" s="22"/>
       <c r="C42" s="6"/>
@@ -5273,7 +5356,7 @@
       <c r="F42" s="24"/>
       <c r="G42" s="24"/>
     </row>
-    <row r="43" spans="1:7" ht="15.75" customHeight="1">
+    <row r="43" spans="1:9" ht="15.75" customHeight="1">
       <c r="A43" s="6"/>
       <c r="B43" s="22"/>
       <c r="C43" s="6"/>
@@ -5282,7 +5365,7 @@
       <c r="F43" s="24"/>
       <c r="G43" s="24"/>
     </row>
-    <row r="44" spans="1:7" ht="15.75" customHeight="1">
+    <row r="44" spans="1:9" ht="15.75" customHeight="1">
       <c r="A44" s="6"/>
       <c r="B44" s="22"/>
       <c r="C44" s="6"/>
@@ -5291,7 +5374,7 @@
       <c r="F44" s="24"/>
       <c r="G44" s="24"/>
     </row>
-    <row r="45" spans="1:7" ht="15.75" customHeight="1">
+    <row r="45" spans="1:9" ht="15.75" customHeight="1">
       <c r="A45" s="6"/>
       <c r="B45" s="22"/>
       <c r="C45" s="6"/>
@@ -5300,7 +5383,7 @@
       <c r="F45" s="24"/>
       <c r="G45" s="24"/>
     </row>
-    <row r="46" spans="1:7" ht="15.75" customHeight="1">
+    <row r="46" spans="1:9" ht="15.75" customHeight="1">
       <c r="A46" s="6"/>
       <c r="B46" s="22"/>
       <c r="C46" s="6"/>
@@ -5309,7 +5392,7 @@
       <c r="F46" s="25"/>
       <c r="G46" s="25"/>
     </row>
-    <row r="47" spans="1:7" ht="15.75" customHeight="1">
+    <row r="47" spans="1:9" ht="15.75" customHeight="1">
       <c r="A47" s="6"/>
       <c r="B47" s="22"/>
       <c r="C47" s="6"/>
@@ -5318,7 +5401,7 @@
       <c r="F47" s="25"/>
       <c r="G47" s="25"/>
     </row>
-    <row r="48" spans="1:7" ht="15.75" customHeight="1">
+    <row r="48" spans="1:9" ht="15.75" customHeight="1">
       <c r="A48" s="6"/>
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>

</xml_diff>